<commit_message>
Replace sample deal with an Indian company
</commit_message>
<xml_diff>
--- a/sample_deal/operating_model.xlsx
+++ b/sample_deal/operating_model.xlsx
@@ -420,7 +420,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Operating model, USD thousands</t>
+          <t>Operating model, INR crore</t>
         </is>
       </c>
     </row>
@@ -432,17 +432,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FY2022</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY24</t>
         </is>
       </c>
     </row>
@@ -453,13 +453,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86174</v>
+        <v>761.23</v>
       </c>
       <c r="C4" t="n">
-        <v>87674</v>
+        <v>795.77</v>
       </c>
       <c r="D4" t="n">
-        <v>100499</v>
+        <v>888.22</v>
       </c>
     </row>
     <row r="5">
@@ -469,29 +469,29 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11984</v>
+        <v>98.81</v>
       </c>
       <c r="C5" t="n">
-        <v>13258</v>
+        <v>105.45</v>
       </c>
       <c r="D5" t="n">
-        <v>15453</v>
+        <v>114.02</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Net income</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6301</v>
+        <v>45.26</v>
       </c>
       <c r="C6" t="n">
-        <v>6762</v>
+        <v>52.58</v>
       </c>
       <c r="D6" t="n">
-        <v>8050</v>
+        <v>46.75</v>
       </c>
     </row>
     <row r="7">
@@ -501,13 +501,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7579</v>
+        <v>59.45</v>
       </c>
       <c r="C7" t="n">
-        <v>6647</v>
+        <v>40.19</v>
       </c>
       <c r="D7" t="n">
-        <v>8161</v>
+        <v>46.5</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>INR crore</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FY2023</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY24</t>
         </is>
       </c>
     </row>
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7183</v>
+        <v>55.94</v>
       </c>
       <c r="C4" t="n">
-        <v>6477</v>
+        <v>34.39</v>
       </c>
     </row>
     <row r="5">
@@ -568,10 +568,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20863</v>
+        <v>198.18</v>
       </c>
       <c r="C5" t="n">
-        <v>27847</v>
+        <v>205.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sample deal regenerated with footnote cases
</commit_message>
<xml_diff>
--- a/sample_deal/operating_model.xlsx
+++ b/sample_deal/operating_model.xlsx
@@ -125,6 +125,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>model owner</author>
+  </authors>
+  <commentList>
+    <comment ref="D7" authorId="0" shapeId="0">
+      <text>
+        <t>Includes capitalised borrowing costs of ₹7.30 Cr.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -453,13 +468,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>761.23</v>
+        <v>760.73</v>
       </c>
       <c r="C4" t="n">
-        <v>795.77</v>
+        <v>822.04</v>
       </c>
       <c r="D4" t="n">
-        <v>888.22</v>
+        <v>888.2</v>
       </c>
     </row>
     <row r="5">
@@ -469,13 +484,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>98.81</v>
+        <v>98.76000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>105.45</v>
+        <v>105.43</v>
       </c>
       <c r="D5" t="n">
-        <v>114.02</v>
+        <v>114.04</v>
       </c>
     </row>
     <row r="6">
@@ -485,13 +500,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45.26</v>
+        <v>45.28</v>
       </c>
       <c r="C6" t="n">
-        <v>52.58</v>
+        <v>52.56</v>
       </c>
       <c r="D6" t="n">
-        <v>46.75</v>
+        <v>46.72</v>
       </c>
     </row>
     <row r="7">
@@ -501,17 +516,18 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>59.45</v>
+        <v>59.48</v>
       </c>
       <c r="C7" t="n">
-        <v>40.19</v>
+        <v>40.21</v>
       </c>
       <c r="D7" t="n">
-        <v>46.5</v>
+        <v>77.23999999999999</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -555,10 +571,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55.94</v>
+        <v>55.92</v>
       </c>
       <c r="C4" t="n">
-        <v>34.39</v>
+        <v>34.37</v>
       </c>
     </row>
     <row r="5">
@@ -568,10 +584,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>198.18</v>
+        <v>198.08</v>
       </c>
       <c r="C5" t="n">
-        <v>205.84</v>
+        <v>223.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>